<commit_message>
chore: update 660 Property Trust valuation example workbook
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/1. VALUATION EXAMPLES/660 Property Trust.xlsx
+++ b/1. VALUATION EXAMPLES/660 Property Trust.xlsx
@@ -1,15 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://anchorpointriskza-my.sharepoint.com/personal/henry_anchorpointrisk_co_za/Documents/Desktop/VS_CODE_REPOSITORY/property-valuations-model/1. VALUATION EXAMPLES/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_6FDF71C5AF4291AEC5A84EC862B30DBD0CD747B0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E59449C5-334D-4BFA-827A-6D4127F0F4A6}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="45" windowWidth="22995" windowHeight="10035"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -178,14 +197,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00_);\(&quot;R&quot;#,##0.00\)"/>
-    <numFmt numFmtId="165" formatCode="&quot;R&quot;\ #,##0"/>
-    <numFmt numFmtId="166" formatCode="&quot;R&quot;#,##0_);\(&quot;R&quot;#,##0\)"/>
-    <numFmt numFmtId="167" formatCode="\R#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="&quot;R&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="&quot;R&quot;#,##0.00_);\(&quot;R&quot;#,##0.00\)"/>
+    <numFmt numFmtId="166" formatCode="&quot;R&quot;\ #,##0"/>
+    <numFmt numFmtId="167" formatCode="&quot;R&quot;#,##0_);\(&quot;R&quot;#,##0\)"/>
+    <numFmt numFmtId="168" formatCode="\R#,##0.00"/>
+    <numFmt numFmtId="169" formatCode="&quot;R&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -195,6 +214,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -869,38 +889,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
@@ -913,9 +932,9 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -925,10 +944,10 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="5" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -943,7 +962,7 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="5" fillId="3" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -958,12 +977,12 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -972,8 +991,8 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="5" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -986,9 +1005,9 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" wrapText="1"/>
     </xf>
@@ -997,7 +1016,7 @@
     </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1008,9 +1027,9 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="5" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1021,10 +1040,9 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1037,13 +1055,13 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1058,7 +1076,7 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="3" fillId="4" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1069,9 +1087,9 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1089,10 +1107,10 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1102,7 +1120,7 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1142,14 +1160,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1187,7 +1208,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1259,7 +1280,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1432,7 +1453,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1456,475 +1477,449 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="130" t="s">
+      <c r="A1" s="128" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="129" t="s">
+      <c r="B1" s="127" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="129"/>
-      <c r="D1" s="129"/>
-      <c r="E1" s="128"/>
-      <c r="F1" s="128"/>
-      <c r="G1" s="128"/>
-      <c r="H1" s="128"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="16"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="125"/>
     </row>
     <row r="2" spans="1:13" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="126" t="s">
+      <c r="A2" s="124" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="124"/>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="125">
+      <c r="B2" s="122"/>
+      <c r="C2" s="122"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="123">
         <v>40721</v>
       </c>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="124"/>
-      <c r="I2" s="123"/>
-      <c r="J2" s="16"/>
+      <c r="F2" s="122"/>
+      <c r="G2" s="122"/>
+      <c r="H2" s="122"/>
+      <c r="I2" s="121"/>
     </row>
     <row r="3" spans="1:13" ht="63.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="122" t="s">
+      <c r="A3" s="120" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="121" t="s">
+      <c r="B3" s="119" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="121" t="s">
+      <c r="C3" s="119" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="121" t="s">
+      <c r="D3" s="119" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="121" t="s">
+      <c r="E3" s="119" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="120" t="s">
+      <c r="F3" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="119" t="s">
+      <c r="G3" s="117" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="118" t="s">
+      <c r="H3" s="116" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="117" t="s">
+      <c r="I3" s="115" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="16"/>
     </row>
     <row r="4" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A4" s="115" t="s">
+      <c r="A4" s="113" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="114" t="s">
+      <c r="B4" s="112" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="113"/>
-      <c r="D4" s="113"/>
-      <c r="E4" s="113"/>
-      <c r="F4" s="113" t="s">
+      <c r="C4" s="111"/>
+      <c r="D4" s="111"/>
+      <c r="E4" s="111"/>
+      <c r="F4" s="111" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="111">
+      <c r="G4" s="109">
         <v>70</v>
       </c>
-      <c r="H4" s="110"/>
-      <c r="I4" s="109">
+      <c r="H4" s="108"/>
+      <c r="I4" s="107">
         <f>G4*F4</f>
         <v>116830</v>
       </c>
-      <c r="J4" s="16"/>
-      <c r="L4" s="98"/>
-      <c r="M4" s="97"/>
+      <c r="L4" s="96"/>
+      <c r="M4" s="95"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="115"/>
-      <c r="B5" s="114"/>
-      <c r="C5" s="113"/>
-      <c r="D5" s="113"/>
-      <c r="E5" s="113"/>
-      <c r="F5" s="116"/>
-      <c r="G5" s="111"/>
-      <c r="H5" s="110"/>
-      <c r="I5" s="109"/>
-      <c r="J5" s="16"/>
-      <c r="L5" s="98"/>
-      <c r="M5" s="97"/>
+      <c r="A5" s="113"/>
+      <c r="B5" s="112"/>
+      <c r="C5" s="111"/>
+      <c r="D5" s="111"/>
+      <c r="E5" s="111"/>
+      <c r="F5" s="114"/>
+      <c r="G5" s="109"/>
+      <c r="H5" s="108"/>
+      <c r="I5" s="107"/>
+      <c r="L5" s="96"/>
+      <c r="M5" s="95"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="115"/>
-      <c r="B6" s="114"/>
-      <c r="C6" s="113"/>
-      <c r="D6" s="113"/>
-      <c r="E6" s="113"/>
-      <c r="F6" s="116"/>
-      <c r="G6" s="111"/>
-      <c r="H6" s="110"/>
-      <c r="I6" s="109"/>
-      <c r="J6" s="16"/>
-      <c r="L6" s="98"/>
-      <c r="M6" s="97"/>
+      <c r="A6" s="113"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="111"/>
+      <c r="E6" s="111"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="109"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="107"/>
+      <c r="L6" s="96"/>
+      <c r="M6" s="95"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="115"/>
-      <c r="B7" s="114"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="111"/>
-      <c r="H7" s="110"/>
-      <c r="I7" s="109"/>
-      <c r="J7" s="16"/>
+      <c r="A7" s="113"/>
+      <c r="B7" s="112"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="111"/>
+      <c r="E7" s="111"/>
+      <c r="F7" s="110"/>
+      <c r="G7" s="109"/>
+      <c r="H7" s="108"/>
+      <c r="I7" s="107"/>
       <c r="K7" s="2"/>
-      <c r="L7" s="98"/>
-      <c r="M7" s="97"/>
+      <c r="L7" s="96"/>
+      <c r="M7" s="95"/>
     </row>
     <row r="8" spans="1:13" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="108"/>
-      <c r="B8" s="81" t="s">
+      <c r="A8" s="106"/>
+      <c r="B8" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="89" t="s">
+      <c r="C8" s="87" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="107" t="s">
+      <c r="D8" s="105" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="107" t="s">
+      <c r="E8" s="105" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="106"/>
-      <c r="G8" s="105"/>
-      <c r="H8" s="104"/>
-      <c r="I8" s="77"/>
-      <c r="J8" s="16"/>
-      <c r="L8" s="98"/>
-      <c r="M8" s="97"/>
+      <c r="F8" s="104"/>
+      <c r="G8" s="103"/>
+      <c r="H8" s="102"/>
+      <c r="I8" s="76"/>
+      <c r="L8" s="96"/>
+      <c r="M8" s="95"/>
     </row>
     <row r="9" spans="1:13" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="103" t="s">
+      <c r="A9" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="102"/>
-      <c r="C9" s="102"/>
-      <c r="D9" s="102"/>
-      <c r="E9" s="102"/>
-      <c r="F9" s="101">
+      <c r="B9" s="100"/>
+      <c r="C9" s="100"/>
+      <c r="D9" s="100"/>
+      <c r="E9" s="100"/>
+      <c r="F9" s="99">
         <v>1669</v>
       </c>
-      <c r="G9" s="100">
+      <c r="G9" s="98">
         <f>I9/F9-H9</f>
         <v>70</v>
       </c>
-      <c r="H9" s="99">
+      <c r="H9" s="97">
         <v>0</v>
       </c>
-      <c r="I9" s="99">
+      <c r="I9" s="97">
         <f>SUM(I4:I8)</f>
         <v>116830</v>
       </c>
-      <c r="J9" s="16"/>
-      <c r="L9" s="98"/>
-      <c r="M9" s="97"/>
+      <c r="L9" s="96"/>
+      <c r="M9" s="95"/>
     </row>
     <row r="10" spans="1:13" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A10" s="96"/>
-      <c r="B10" s="95"/>
-      <c r="C10" s="95"/>
-      <c r="D10" s="95"/>
-      <c r="E10" s="94"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="92"/>
-      <c r="H10" s="78"/>
-      <c r="I10" s="77"/>
-      <c r="J10" s="16"/>
+      <c r="A10" s="94"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="92"/>
+      <c r="F10" s="91"/>
+      <c r="G10" s="90"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="76"/>
     </row>
     <row r="11" spans="1:13" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="91" t="s">
+      <c r="A11" s="89" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="90"/>
-      <c r="C11" s="90"/>
-      <c r="D11" s="90"/>
-      <c r="E11" s="89"/>
-      <c r="F11" s="88" t="s">
+      <c r="B11" s="88"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="87"/>
+      <c r="F11" s="86" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="87" t="s">
+      <c r="G11" s="85" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="78"/>
-      <c r="I11" s="77"/>
-      <c r="J11" s="16"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="76"/>
     </row>
     <row r="12" spans="1:13" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="86"/>
-      <c r="B12" s="85"/>
-      <c r="C12" s="85"/>
-      <c r="D12" s="85"/>
-      <c r="E12" s="84"/>
-      <c r="F12" s="80"/>
-      <c r="G12" s="79"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="77"/>
-      <c r="J12" s="16"/>
+      <c r="A12" s="84"/>
+      <c r="B12" s="83"/>
+      <c r="C12" s="83"/>
+      <c r="D12" s="83"/>
+      <c r="E12" s="82"/>
+      <c r="F12" s="78"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="76"/>
     </row>
     <row r="13" spans="1:13" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="86"/>
-      <c r="B13" s="85"/>
-      <c r="C13" s="85"/>
-      <c r="D13" s="85"/>
-      <c r="E13" s="84"/>
-      <c r="F13" s="80"/>
-      <c r="G13" s="79"/>
-      <c r="H13" s="78"/>
-      <c r="I13" s="77"/>
-      <c r="J13" s="16"/>
+      <c r="A13" s="84"/>
+      <c r="B13" s="83"/>
+      <c r="C13" s="83"/>
+      <c r="D13" s="83"/>
+      <c r="E13" s="82"/>
+      <c r="F13" s="78"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="76"/>
     </row>
     <row r="14" spans="1:13" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A14" s="86"/>
-      <c r="B14" s="85"/>
-      <c r="C14" s="85"/>
-      <c r="D14" s="85"/>
-      <c r="E14" s="84" t="s">
+      <c r="A14" s="84"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="83"/>
+      <c r="D14" s="83"/>
+      <c r="E14" s="82" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="80">
+      <c r="F14" s="78">
         <v>0</v>
       </c>
-      <c r="G14" s="79">
+      <c r="G14" s="77">
         <v>0</v>
       </c>
-      <c r="H14" s="78"/>
-      <c r="I14" s="77">
+      <c r="H14" s="13"/>
+      <c r="I14" s="76">
         <f>G14*F14</f>
         <v>0</v>
       </c>
-      <c r="J14" s="16"/>
     </row>
     <row r="15" spans="1:13" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="83"/>
-      <c r="B15" s="82"/>
-      <c r="C15" s="82"/>
-      <c r="D15" s="82"/>
-      <c r="E15" s="81"/>
-      <c r="F15" s="80"/>
-      <c r="G15" s="79"/>
-      <c r="H15" s="78"/>
-      <c r="I15" s="77">
+      <c r="A15" s="81"/>
+      <c r="B15" s="80"/>
+      <c r="C15" s="80"/>
+      <c r="D15" s="80"/>
+      <c r="E15" s="79"/>
+      <c r="F15" s="78"/>
+      <c r="G15" s="77"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="76">
         <f>G15*F15</f>
         <v>0</v>
       </c>
-      <c r="J15" s="16"/>
     </row>
     <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="76" t="s">
+      <c r="A16" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="75"/>
-      <c r="C16" s="75"/>
-      <c r="D16" s="75"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="73">
+      <c r="B16" s="74"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="73"/>
+      <c r="F16" s="72">
         <f>SUM(F12:F15)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="72"/>
-      <c r="H16" s="71"/>
-      <c r="I16" s="70">
+      <c r="G16" s="71"/>
+      <c r="H16" s="70"/>
+      <c r="I16" s="69">
         <f>SUM(I12:I15)</f>
         <v>0</v>
       </c>
-      <c r="J16" s="16"/>
     </row>
     <row r="17" spans="1:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="69" t="s">
+      <c r="A17" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="68"/>
-      <c r="C17" s="68"/>
-      <c r="D17" s="68"/>
-      <c r="E17" s="67"/>
-      <c r="F17" s="66"/>
-      <c r="G17" s="65"/>
-      <c r="H17" s="60"/>
-      <c r="I17" s="58">
+      <c r="B17" s="67"/>
+      <c r="C17" s="67"/>
+      <c r="D17" s="67"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="65"/>
+      <c r="G17" s="64"/>
+      <c r="H17" s="59"/>
+      <c r="I17" s="57">
         <f>+I16+I9</f>
         <v>116830</v>
       </c>
-      <c r="J17" s="16"/>
     </row>
     <row r="18" spans="1:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="64" t="s">
+      <c r="A18" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="60"/>
-      <c r="H18" s="59"/>
-      <c r="I18" s="58">
+      <c r="B18" s="62"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="62"/>
+      <c r="E18" s="61"/>
+      <c r="F18" s="60"/>
+      <c r="G18" s="59"/>
+      <c r="H18" s="58"/>
+      <c r="I18" s="57">
         <f>+I17*12</f>
         <v>1401960</v>
       </c>
-      <c r="J18" s="16"/>
     </row>
     <row r="19" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="57" t="s">
+      <c r="A19" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="56"/>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="55" t="s">
+      <c r="B19" s="55"/>
+      <c r="C19" s="55"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="F19" s="55" t="s">
+      <c r="F19" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="G19" s="54" t="s">
+      <c r="G19" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="H19" s="53"/>
-      <c r="I19" s="52"/>
-      <c r="J19" s="16"/>
+      <c r="H19" s="52"/>
+      <c r="I19" s="51"/>
     </row>
     <row r="20" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="51" t="s">
+      <c r="A20" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="50"/>
-      <c r="C20" s="50"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="49">
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="48">
         <v>18097.25</v>
       </c>
-      <c r="F20" s="49">
+      <c r="F20" s="48">
         <f>E20*12</f>
         <v>217167</v>
       </c>
-      <c r="G20" s="48">
+      <c r="G20" s="47">
         <f>E20/F9</f>
         <v>10.843169562612342</v>
       </c>
-      <c r="H20" s="47">
+      <c r="H20" s="46">
         <f>F20/I18</f>
         <v>0.15490242232303347</v>
       </c>
-      <c r="I20" s="46"/>
-      <c r="J20" s="16"/>
+      <c r="I20" s="45"/>
     </row>
     <row r="21" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="45" t="s">
+      <c r="A21" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="44"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="40">
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="39">
         <v>0.01</v>
       </c>
-      <c r="I21" s="39">
+      <c r="I21" s="38">
         <f>+I18*-H21</f>
         <v>-14019.6</v>
       </c>
-      <c r="J21" s="16"/>
     </row>
     <row r="22" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="38" t="s">
+      <c r="A22" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="32">
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="31">
         <f>+I23/12</f>
         <v>97564.45</v>
       </c>
-      <c r="J22" s="16"/>
     </row>
     <row r="23" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="29">
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="28">
         <f>+I18-F20+I21</f>
         <v>1170773.3999999999</v>
       </c>
-      <c r="J23" s="16"/>
     </row>
     <row r="24" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="24">
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="23">
         <v>0.12</v>
       </c>
-      <c r="I24" s="29">
+      <c r="I24" s="28">
         <f>+I23/H24</f>
         <v>9756445</v>
       </c>
-      <c r="J24" s="16"/>
     </row>
     <row r="25" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="23">
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="22">
         <f>ROUND(I24,-4)</f>
         <v>9760000</v>
       </c>
-      <c r="J25" s="16"/>
     </row>
     <row r="26" spans="1:12" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="22"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="17">
+      <c r="A26" s="21"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="16">
         <f>L26/I25</f>
         <v>0.29607758299180326</v>
       </c>
-      <c r="J26" s="16"/>
       <c r="L26" s="15">
         <v>2889717.21</v>
       </c>

</xml_diff>